<commit_message>
inventario: 178 productos disponibles (2026-05-18)
</commit_message>
<xml_diff>
--- a/assets/LISTA ZAPATILLAS.xlsx
+++ b/assets/LISTA ZAPATILLAS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8bfe2c87cad12b0/IA/MILENASHOES/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="79" documentId="13_ncr:1_{E0C42F5F-A3E4-4F22-AD40-E0497D996882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BCA1ACB4-A517-45A0-B9B2-5B5BEBAE0C1E}"/>
+  <xr:revisionPtr revIDLastSave="82" documentId="13_ncr:1_{E0C42F5F-A3E4-4F22-AD40-E0497D996882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{20CDAEAB-ACCB-4C46-80BF-65540EB42DE1}"/>
   <bookViews>
     <workbookView xWindow="1545" yWindow="1125" windowWidth="15570" windowHeight="13710" xr2:uid="{B7A6A16F-7A19-4864-8939-1CF29A8D65F8}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="INVENTARIO" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">INVENTARIO!$B$2:$I$180</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">INVENTARIO!$B$2:$I$192</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -30,9 +30,10 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -447,7 +448,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -595,7 +596,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -892,7 +893,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F75DB620-AF17-408B-81D4-431B9D551CF9}">
   <dimension ref="B2:I193"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.42578125" customWidth="1"/>
     <col min="2" max="2" width="14.28515625" style="7" bestFit="1" customWidth="1"/>
@@ -904,7 +905,7 @@
     <col min="9" max="9" width="16" style="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>0</v>
       </c>
@@ -930,7 +931,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="2:9">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="5">
         <v>1</v>
       </c>
@@ -957,7 +958,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="2:9">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="5">
         <v>2</v>
       </c>
@@ -984,7 +985,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:9">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="5">
         <v>3</v>
       </c>
@@ -1011,7 +1012,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:9">
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B6" s="5">
         <v>4</v>
       </c>
@@ -1038,7 +1039,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="2:9">
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B7" s="5">
         <v>5</v>
       </c>
@@ -1065,7 +1066,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="2:9">
+    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B8" s="5">
         <v>6</v>
       </c>
@@ -1092,7 +1093,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="2:9">
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B9" s="5">
         <v>7</v>
       </c>
@@ -1119,7 +1120,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="2:9">
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" s="5">
         <v>8</v>
       </c>
@@ -1146,7 +1147,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="2:9">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B11" s="5">
         <v>9</v>
       </c>
@@ -1173,7 +1174,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="2:9">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" s="5">
         <v>10</v>
       </c>
@@ -1200,7 +1201,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="2:9">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="5">
         <v>11</v>
       </c>
@@ -1227,7 +1228,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="2:9">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="5">
         <v>12</v>
       </c>
@@ -1254,7 +1255,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="2:9">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B15" s="5">
         <v>13</v>
       </c>
@@ -1281,7 +1282,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="2:9">
+    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B16" s="5">
         <v>14</v>
       </c>
@@ -1308,7 +1309,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="2:9">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B17" s="5">
         <v>15</v>
       </c>
@@ -1335,7 +1336,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="2:9">
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B18" s="5">
         <v>16</v>
       </c>
@@ -1362,7 +1363,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="2:9">
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B19" s="5">
         <v>17</v>
       </c>
@@ -1389,7 +1390,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="2:9">
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B20" s="5">
         <v>18</v>
       </c>
@@ -1416,7 +1417,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="2:9">
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B21" s="5">
         <v>19</v>
       </c>
@@ -1443,7 +1444,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="2:9">
+    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B22" s="5">
         <v>20</v>
       </c>
@@ -1470,7 +1471,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="2:9">
+    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B23" s="5">
         <v>21</v>
       </c>
@@ -1497,7 +1498,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="2:9">
+    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B24" s="5">
         <v>22</v>
       </c>
@@ -1524,7 +1525,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="25" spans="2:9">
+    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B25" s="5">
         <v>23</v>
       </c>
@@ -1551,7 +1552,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="26" spans="2:9">
+    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B26" s="5">
         <v>24</v>
       </c>
@@ -1559,7 +1560,7 @@
         <v>13</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>37</v>
@@ -1578,7 +1579,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="2:9">
+    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B27" s="5">
         <v>25</v>
       </c>
@@ -1605,7 +1606,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="2:9">
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B28" s="5">
         <v>26</v>
       </c>
@@ -1632,7 +1633,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="29" spans="2:9">
+    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B29" s="5">
         <v>27</v>
       </c>
@@ -1659,7 +1660,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="2:9">
+    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B30" s="5">
         <v>28</v>
       </c>
@@ -1686,7 +1687,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="31" spans="2:9">
+    <row r="31" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B31" s="5">
         <v>29</v>
       </c>
@@ -1713,7 +1714,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="32" spans="2:9">
+    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B32" s="5">
         <v>30</v>
       </c>
@@ -1740,7 +1741,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="33" spans="2:9">
+    <row r="33" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B33" s="5">
         <v>31</v>
       </c>
@@ -1767,7 +1768,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="34" spans="2:9">
+    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B34" s="5">
         <v>32</v>
       </c>
@@ -1794,7 +1795,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="35" spans="2:9">
+    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B35" s="5">
         <v>33</v>
       </c>
@@ -1821,7 +1822,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="36" spans="2:9">
+    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B36" s="5">
         <v>34</v>
       </c>
@@ -1848,7 +1849,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="37" spans="2:9">
+    <row r="37" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B37" s="5">
         <v>35</v>
       </c>
@@ -1875,7 +1876,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="38" spans="2:9">
+    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B38" s="5">
         <v>36</v>
       </c>
@@ -1902,7 +1903,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="39" spans="2:9">
+    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B39" s="5">
         <v>37</v>
       </c>
@@ -1929,7 +1930,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="40" spans="2:9">
+    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B40" s="5">
         <v>38</v>
       </c>
@@ -1956,7 +1957,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="41" spans="2:9">
+    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B41" s="5">
         <v>39</v>
       </c>
@@ -1983,7 +1984,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="42" spans="2:9">
+    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B42" s="5">
         <v>40</v>
       </c>
@@ -2010,7 +2011,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="43" spans="2:9">
+    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B43" s="5">
         <v>41</v>
       </c>
@@ -2037,7 +2038,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="44" spans="2:9">
+    <row r="44" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B44" s="5">
         <v>42</v>
       </c>
@@ -2064,7 +2065,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="45" spans="2:9">
+    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B45" s="5">
         <v>43</v>
       </c>
@@ -2091,7 +2092,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="46" spans="2:9">
+    <row r="46" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B46" s="5">
         <v>44</v>
       </c>
@@ -2118,7 +2119,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="47" spans="2:9">
+    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B47" s="5">
         <v>45</v>
       </c>
@@ -2145,7 +2146,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="48" spans="2:9">
+    <row r="48" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B48" s="5">
         <v>46</v>
       </c>
@@ -2172,7 +2173,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="49" spans="2:9">
+    <row r="49" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B49" s="5">
         <v>47</v>
       </c>
@@ -2199,7 +2200,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="50" spans="2:9">
+    <row r="50" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B50" s="5">
         <v>48</v>
       </c>
@@ -2226,7 +2227,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="51" spans="2:9">
+    <row r="51" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B51" s="5">
         <v>49</v>
       </c>
@@ -2253,7 +2254,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="52" spans="2:9">
+    <row r="52" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B52" s="5">
         <v>50</v>
       </c>
@@ -2280,7 +2281,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="53" spans="2:9">
+    <row r="53" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B53" s="5">
         <v>51</v>
       </c>
@@ -2307,7 +2308,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="54" spans="2:9">
+    <row r="54" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B54" s="5">
         <v>52</v>
       </c>
@@ -2334,7 +2335,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="55" spans="2:9">
+    <row r="55" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B55" s="5">
         <v>53</v>
       </c>
@@ -2361,7 +2362,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="56" spans="2:9">
+    <row r="56" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B56" s="5">
         <v>54</v>
       </c>
@@ -2388,7 +2389,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="57" spans="2:9">
+    <row r="57" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B57" s="5">
         <v>55</v>
       </c>
@@ -2415,7 +2416,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="58" spans="2:9">
+    <row r="58" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B58" s="5">
         <v>56</v>
       </c>
@@ -2442,7 +2443,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="59" spans="2:9">
+    <row r="59" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B59" s="5">
         <v>57</v>
       </c>
@@ -2469,7 +2470,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="60" spans="2:9">
+    <row r="60" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B60" s="5">
         <v>58</v>
       </c>
@@ -2496,7 +2497,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="61" spans="2:9">
+    <row r="61" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B61" s="5">
         <v>59</v>
       </c>
@@ -2523,7 +2524,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="62" spans="2:9">
+    <row r="62" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B62" s="5">
         <v>60</v>
       </c>
@@ -2550,7 +2551,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="63" spans="2:9">
+    <row r="63" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B63" s="5">
         <v>61</v>
       </c>
@@ -2577,7 +2578,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="64" spans="2:9">
+    <row r="64" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B64" s="5">
         <v>62</v>
       </c>
@@ -2604,7 +2605,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="65" spans="2:9">
+    <row r="65" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B65" s="5">
         <v>63</v>
       </c>
@@ -2631,7 +2632,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="66" spans="2:9">
+    <row r="66" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B66" s="5">
         <v>64</v>
       </c>
@@ -2658,7 +2659,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="67" spans="2:9">
+    <row r="67" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B67" s="5">
         <v>65</v>
       </c>
@@ -2685,7 +2686,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="68" spans="2:9">
+    <row r="68" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B68" s="5">
         <v>66</v>
       </c>
@@ -2712,7 +2713,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="69" spans="2:9">
+    <row r="69" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B69" s="5">
         <v>67</v>
       </c>
@@ -2739,7 +2740,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="70" spans="2:9">
+    <row r="70" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B70" s="5">
         <v>68</v>
       </c>
@@ -2766,7 +2767,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="71" spans="2:9">
+    <row r="71" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B71" s="5">
         <v>69</v>
       </c>
@@ -2793,7 +2794,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="72" spans="2:9">
+    <row r="72" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B72" s="5">
         <v>70</v>
       </c>
@@ -2820,7 +2821,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="73" spans="2:9">
+    <row r="73" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B73" s="5">
         <v>71</v>
       </c>
@@ -2847,7 +2848,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="74" spans="2:9">
+    <row r="74" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B74" s="5">
         <v>72</v>
       </c>
@@ -2874,7 +2875,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="75" spans="2:9">
+    <row r="75" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B75" s="5">
         <v>73</v>
       </c>
@@ -2901,7 +2902,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="76" spans="2:9">
+    <row r="76" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B76" s="5">
         <v>74</v>
       </c>
@@ -2928,7 +2929,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="77" spans="2:9">
+    <row r="77" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B77" s="5">
         <v>75</v>
       </c>
@@ -2955,7 +2956,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="78" spans="2:9">
+    <row r="78" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B78" s="5">
         <v>76</v>
       </c>
@@ -2982,7 +2983,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="79" spans="2:9">
+    <row r="79" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B79" s="5">
         <v>77</v>
       </c>
@@ -3009,7 +3010,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="80" spans="2:9">
+    <row r="80" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B80" s="5">
         <v>78</v>
       </c>
@@ -3036,7 +3037,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="81" spans="2:9">
+    <row r="81" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B81" s="5">
         <v>79</v>
       </c>
@@ -3063,7 +3064,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="82" spans="2:9">
+    <row r="82" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B82" s="5">
         <v>80</v>
       </c>
@@ -3090,7 +3091,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="83" spans="2:9">
+    <row r="83" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B83" s="5">
         <v>81</v>
       </c>
@@ -3117,7 +3118,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="84" spans="2:9">
+    <row r="84" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B84" s="5">
         <v>82</v>
       </c>
@@ -3144,7 +3145,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="85" spans="2:9">
+    <row r="85" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B85" s="5">
         <v>83</v>
       </c>
@@ -3171,7 +3172,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="86" spans="2:9">
+    <row r="86" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B86" s="5">
         <v>84</v>
       </c>
@@ -3198,7 +3199,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="87" spans="2:9">
+    <row r="87" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B87" s="5">
         <v>85</v>
       </c>
@@ -3225,7 +3226,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="88" spans="2:9">
+    <row r="88" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B88" s="5">
         <v>86</v>
       </c>
@@ -3252,7 +3253,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="89" spans="2:9">
+    <row r="89" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B89" s="5">
         <v>87</v>
       </c>
@@ -3279,7 +3280,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="90" spans="2:9">
+    <row r="90" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B90" s="5">
         <v>88</v>
       </c>
@@ -3306,7 +3307,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="91" spans="2:9">
+    <row r="91" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B91" s="5">
         <v>89</v>
       </c>
@@ -3333,7 +3334,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="92" spans="2:9">
+    <row r="92" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B92" s="5">
         <v>90</v>
       </c>
@@ -3360,7 +3361,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="93" spans="2:9">
+    <row r="93" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B93" s="5">
         <v>91</v>
       </c>
@@ -3387,7 +3388,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="94" spans="2:9">
+    <row r="94" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B94" s="5">
         <v>92</v>
       </c>
@@ -3414,7 +3415,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="95" spans="2:9">
+    <row r="95" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B95" s="5">
         <v>93</v>
       </c>
@@ -3441,7 +3442,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="96" spans="2:9">
+    <row r="96" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B96" s="5">
         <v>94</v>
       </c>
@@ -3468,7 +3469,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="97" spans="2:9">
+    <row r="97" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B97" s="5">
         <v>95</v>
       </c>
@@ -3495,7 +3496,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="98" spans="2:9">
+    <row r="98" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B98" s="5">
         <v>96</v>
       </c>
@@ -3522,7 +3523,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="99" spans="2:9">
+    <row r="99" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B99" s="5">
         <v>97</v>
       </c>
@@ -3549,7 +3550,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="100" spans="2:9">
+    <row r="100" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B100" s="5">
         <v>98</v>
       </c>
@@ -3576,7 +3577,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="101" spans="2:9">
+    <row r="101" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B101" s="5">
         <v>99</v>
       </c>
@@ -3603,7 +3604,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="102" spans="2:9">
+    <row r="102" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B102" s="5">
         <v>100</v>
       </c>
@@ -3630,7 +3631,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="103" spans="2:9">
+    <row r="103" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B103" s="5">
         <v>101</v>
       </c>
@@ -3657,7 +3658,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="104" spans="2:9">
+    <row r="104" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B104" s="5">
         <v>102</v>
       </c>
@@ -3684,7 +3685,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="105" spans="2:9">
+    <row r="105" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B105" s="5">
         <v>103</v>
       </c>
@@ -3711,7 +3712,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="106" spans="2:9">
+    <row r="106" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B106" s="5">
         <v>104</v>
       </c>
@@ -3738,7 +3739,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="107" spans="2:9">
+    <row r="107" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B107" s="5">
         <v>105</v>
       </c>
@@ -3765,7 +3766,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="108" spans="2:9">
+    <row r="108" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B108" s="5">
         <v>106</v>
       </c>
@@ -3792,7 +3793,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="109" spans="2:9">
+    <row r="109" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B109" s="5">
         <v>107</v>
       </c>
@@ -3819,7 +3820,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="110" spans="2:9">
+    <row r="110" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B110" s="5">
         <v>108</v>
       </c>
@@ -3846,7 +3847,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="111" spans="2:9">
+    <row r="111" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B111" s="5">
         <v>109</v>
       </c>
@@ -3873,7 +3874,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="112" spans="2:9">
+    <row r="112" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B112" s="5">
         <v>110</v>
       </c>
@@ -3900,7 +3901,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="113" spans="2:9">
+    <row r="113" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B113" s="5">
         <v>111</v>
       </c>
@@ -3927,7 +3928,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="114" spans="2:9">
+    <row r="114" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B114" s="5">
         <v>112</v>
       </c>
@@ -3954,7 +3955,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="115" spans="2:9">
+    <row r="115" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B115" s="5">
         <v>113</v>
       </c>
@@ -3981,7 +3982,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="116" spans="2:9">
+    <row r="116" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B116" s="5">
         <v>114</v>
       </c>
@@ -4008,7 +4009,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="117" spans="2:9">
+    <row r="117" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B117" s="5">
         <v>115</v>
       </c>
@@ -4035,7 +4036,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="118" spans="2:9">
+    <row r="118" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B118" s="5">
         <v>116</v>
       </c>
@@ -4062,7 +4063,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="119" spans="2:9">
+    <row r="119" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B119" s="5">
         <v>117</v>
       </c>
@@ -4089,7 +4090,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="120" spans="2:9">
+    <row r="120" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B120" s="5">
         <v>118</v>
       </c>
@@ -4116,7 +4117,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="121" spans="2:9">
+    <row r="121" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B121" s="5">
         <v>119</v>
       </c>
@@ -4143,7 +4144,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="122" spans="2:9">
+    <row r="122" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B122" s="5">
         <v>120</v>
       </c>
@@ -4170,7 +4171,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="123" spans="2:9">
+    <row r="123" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B123" s="5">
         <v>121</v>
       </c>
@@ -4197,7 +4198,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="124" spans="2:9">
+    <row r="124" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B124" s="5">
         <v>122</v>
       </c>
@@ -4224,7 +4225,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="125" spans="2:9">
+    <row r="125" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B125" s="5">
         <v>123</v>
       </c>
@@ -4251,7 +4252,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="126" spans="2:9">
+    <row r="126" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B126" s="5">
         <v>124</v>
       </c>
@@ -4278,7 +4279,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="127" spans="2:9">
+    <row r="127" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B127" s="5">
         <v>125</v>
       </c>
@@ -4305,7 +4306,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="128" spans="2:9">
+    <row r="128" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B128" s="6">
         <v>126</v>
       </c>
@@ -4332,7 +4333,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="129" spans="2:9">
+    <row r="129" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B129" s="6">
         <v>127</v>
       </c>
@@ -4359,7 +4360,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="130" spans="2:9">
+    <row r="130" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B130" s="6">
         <v>128</v>
       </c>
@@ -4386,7 +4387,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="131" spans="2:9">
+    <row r="131" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B131" s="6">
         <v>129</v>
       </c>
@@ -4413,7 +4414,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="132" spans="2:9">
+    <row r="132" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B132" s="6">
         <v>130</v>
       </c>
@@ -4440,7 +4441,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="133" spans="2:9">
+    <row r="133" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B133" s="6">
         <v>131</v>
       </c>
@@ -4467,7 +4468,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="134" spans="2:9">
+    <row r="134" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B134" s="6">
         <v>132</v>
       </c>
@@ -4494,7 +4495,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="135" spans="2:9">
+    <row r="135" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B135" s="6">
         <v>133</v>
       </c>
@@ -4521,7 +4522,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="136" spans="2:9">
+    <row r="136" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B136" s="6">
         <v>134</v>
       </c>
@@ -4548,7 +4549,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="137" spans="2:9">
+    <row r="137" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B137" s="6">
         <v>135</v>
       </c>
@@ -4575,7 +4576,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="138" spans="2:9">
+    <row r="138" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B138" s="6">
         <v>136</v>
       </c>
@@ -4602,7 +4603,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="139" spans="2:9">
+    <row r="139" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B139" s="6">
         <v>137</v>
       </c>
@@ -4629,7 +4630,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="140" spans="2:9">
+    <row r="140" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B140" s="6">
         <v>138</v>
       </c>
@@ -4656,7 +4657,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="141" spans="2:9">
+    <row r="141" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B141" s="6">
         <v>139</v>
       </c>
@@ -4683,7 +4684,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="142" spans="2:9">
+    <row r="142" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B142" s="6">
         <v>140</v>
       </c>
@@ -4710,7 +4711,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="143" spans="2:9">
+    <row r="143" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B143" s="6">
         <v>141</v>
       </c>
@@ -4737,7 +4738,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="144" spans="2:9">
+    <row r="144" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B144" s="6">
         <v>142</v>
       </c>
@@ -4764,7 +4765,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="145" spans="2:9">
+    <row r="145" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B145" s="6">
         <v>143</v>
       </c>
@@ -4791,7 +4792,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="146" spans="2:9">
+    <row r="146" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B146" s="6">
         <v>144</v>
       </c>
@@ -4818,7 +4819,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="147" spans="2:9">
+    <row r="147" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B147" s="6">
         <v>145</v>
       </c>
@@ -4845,7 +4846,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="148" spans="2:9">
+    <row r="148" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B148" s="6">
         <v>146</v>
       </c>
@@ -4872,7 +4873,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="149" spans="2:9">
+    <row r="149" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B149" s="6">
         <v>147</v>
       </c>
@@ -4899,7 +4900,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="150" spans="2:9">
+    <row r="150" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B150" s="6">
         <v>148</v>
       </c>
@@ -4926,7 +4927,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="151" spans="2:9">
+    <row r="151" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B151" s="6">
         <v>149</v>
       </c>
@@ -4953,7 +4954,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="152" spans="2:9">
+    <row r="152" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B152" s="6">
         <v>150</v>
       </c>
@@ -4980,7 +4981,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="153" spans="2:9">
+    <row r="153" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B153" s="6">
         <v>151</v>
       </c>
@@ -5007,7 +5008,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="154" spans="2:9">
+    <row r="154" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B154" s="6">
         <v>152</v>
       </c>
@@ -5034,7 +5035,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="155" spans="2:9">
+    <row r="155" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B155" s="6">
         <v>153</v>
       </c>
@@ -5061,7 +5062,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="156" spans="2:9">
+    <row r="156" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B156" s="6">
         <v>154</v>
       </c>
@@ -5088,7 +5089,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="157" spans="2:9">
+    <row r="157" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B157" s="6">
         <v>155</v>
       </c>
@@ -5115,7 +5116,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="158" spans="2:9">
+    <row r="158" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B158" s="6">
         <v>156</v>
       </c>
@@ -5142,7 +5143,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="159" spans="2:9">
+    <row r="159" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B159" s="8">
         <v>157</v>
       </c>
@@ -5169,7 +5170,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="160" spans="2:9">
+    <row r="160" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B160" s="6">
         <v>158</v>
       </c>
@@ -5194,7 +5195,7 @@
       </c>
       <c r="I160" s="6"/>
     </row>
-    <row r="161" spans="2:9">
+    <row r="161" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B161" s="6">
         <v>159</v>
       </c>
@@ -5219,7 +5220,7 @@
       </c>
       <c r="I161" s="6"/>
     </row>
-    <row r="162" spans="2:9">
+    <row r="162" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B162" s="6">
         <v>160</v>
       </c>
@@ -5244,7 +5245,7 @@
       </c>
       <c r="I162" s="6"/>
     </row>
-    <row r="163" spans="2:9">
+    <row r="163" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B163" s="6">
         <v>161</v>
       </c>
@@ -5269,7 +5270,7 @@
       </c>
       <c r="I163" s="6"/>
     </row>
-    <row r="164" spans="2:9">
+    <row r="164" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B164" s="6">
         <v>162</v>
       </c>
@@ -5294,7 +5295,7 @@
       </c>
       <c r="I164" s="6"/>
     </row>
-    <row r="165" spans="2:9">
+    <row r="165" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B165" s="6">
         <v>163</v>
       </c>
@@ -5319,7 +5320,7 @@
       </c>
       <c r="I165" s="6"/>
     </row>
-    <row r="166" spans="2:9">
+    <row r="166" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B166" s="6">
         <v>164</v>
       </c>
@@ -5344,7 +5345,7 @@
       </c>
       <c r="I166" s="6"/>
     </row>
-    <row r="167" spans="2:9">
+    <row r="167" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B167" s="6">
         <v>165</v>
       </c>
@@ -5369,7 +5370,7 @@
       </c>
       <c r="I167" s="6"/>
     </row>
-    <row r="168" spans="2:9">
+    <row r="168" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B168" s="6">
         <v>166</v>
       </c>
@@ -5394,7 +5395,7 @@
       </c>
       <c r="I168" s="6"/>
     </row>
-    <row r="169" spans="2:9">
+    <row r="169" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B169" s="6">
         <v>167</v>
       </c>
@@ -5419,7 +5420,7 @@
       </c>
       <c r="I169" s="6"/>
     </row>
-    <row r="170" spans="2:9">
+    <row r="170" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B170" s="6">
         <v>168</v>
       </c>
@@ -5444,7 +5445,7 @@
       </c>
       <c r="I170" s="6"/>
     </row>
-    <row r="171" spans="2:9">
+    <row r="171" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B171" s="6">
         <v>169</v>
       </c>
@@ -5469,7 +5470,7 @@
       </c>
       <c r="I171" s="6"/>
     </row>
-    <row r="172" spans="2:9">
+    <row r="172" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B172" s="6">
         <v>170</v>
       </c>
@@ -5494,7 +5495,7 @@
       </c>
       <c r="I172" s="6"/>
     </row>
-    <row r="173" spans="2:9">
+    <row r="173" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B173" s="6">
         <v>171</v>
       </c>
@@ -5519,7 +5520,7 @@
       </c>
       <c r="I173" s="6"/>
     </row>
-    <row r="174" spans="2:9">
+    <row r="174" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B174" s="6">
         <v>172</v>
       </c>
@@ -5544,7 +5545,7 @@
       </c>
       <c r="I174" s="6"/>
     </row>
-    <row r="175" spans="2:9">
+    <row r="175" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B175" s="6">
         <v>173</v>
       </c>
@@ -5569,7 +5570,7 @@
       </c>
       <c r="I175" s="6"/>
     </row>
-    <row r="176" spans="2:9">
+    <row r="176" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B176" s="6">
         <v>174</v>
       </c>
@@ -5594,7 +5595,7 @@
       </c>
       <c r="I176" s="6"/>
     </row>
-    <row r="177" spans="2:9">
+    <row r="177" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B177" s="6">
         <v>175</v>
       </c>
@@ -5619,7 +5620,7 @@
       </c>
       <c r="I177" s="6"/>
     </row>
-    <row r="178" spans="2:9" s="19" customFormat="1">
+    <row r="178" spans="2:9" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B178" s="15">
         <v>176</v>
       </c>
@@ -5644,7 +5645,7 @@
       </c>
       <c r="I178" s="15"/>
     </row>
-    <row r="179" spans="2:9">
+    <row r="179" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B179" s="6">
         <v>177</v>
       </c>
@@ -5669,7 +5670,7 @@
       </c>
       <c r="I179" s="6"/>
     </row>
-    <row r="180" spans="2:9">
+    <row r="180" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B180" s="6">
         <v>178</v>
       </c>
@@ -5694,7 +5695,7 @@
       </c>
       <c r="I180" s="6"/>
     </row>
-    <row r="181" spans="2:9" s="23" customFormat="1">
+    <row r="181" spans="2:9" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B181" s="6">
         <v>179</v>
       </c>
@@ -5719,7 +5720,7 @@
       </c>
       <c r="I181" s="6"/>
     </row>
-    <row r="182" spans="2:9">
+    <row r="182" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B182" s="6">
         <v>180</v>
       </c>
@@ -5744,7 +5745,7 @@
       </c>
       <c r="I182" s="6"/>
     </row>
-    <row r="183" spans="2:9">
+    <row r="183" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B183" s="6">
         <v>181</v>
       </c>
@@ -5769,7 +5770,7 @@
       </c>
       <c r="I183" s="6"/>
     </row>
-    <row r="184" spans="2:9">
+    <row r="184" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B184" s="6">
         <v>182</v>
       </c>
@@ -5794,7 +5795,7 @@
       </c>
       <c r="I184" s="6"/>
     </row>
-    <row r="185" spans="2:9">
+    <row r="185" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B185" s="6">
         <v>183</v>
       </c>
@@ -5819,7 +5820,7 @@
       </c>
       <c r="I185" s="6"/>
     </row>
-    <row r="186" spans="2:9">
+    <row r="186" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B186" s="6">
         <v>184</v>
       </c>
@@ -5844,7 +5845,7 @@
       </c>
       <c r="I186" s="6"/>
     </row>
-    <row r="187" spans="2:9">
+    <row r="187" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B187" s="6">
         <v>185</v>
       </c>
@@ -5869,7 +5870,7 @@
       </c>
       <c r="I187" s="6"/>
     </row>
-    <row r="188" spans="2:9">
+    <row r="188" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B188" s="6"/>
       <c r="C188" s="5"/>
       <c r="D188" s="13"/>
@@ -5882,7 +5883,7 @@
       </c>
       <c r="I188" s="6"/>
     </row>
-    <row r="189" spans="2:9">
+    <row r="189" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B189" s="6"/>
       <c r="C189" s="5"/>
       <c r="D189" s="13"/>
@@ -5895,7 +5896,7 @@
       </c>
       <c r="I189" s="6"/>
     </row>
-    <row r="190" spans="2:9">
+    <row r="190" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B190" s="6"/>
       <c r="C190" s="5"/>
       <c r="D190" s="13"/>
@@ -5908,7 +5909,7 @@
       </c>
       <c r="I190" s="6"/>
     </row>
-    <row r="191" spans="2:9">
+    <row r="191" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B191" s="6"/>
       <c r="C191" s="5"/>
       <c r="D191" s="13"/>
@@ -5921,7 +5922,7 @@
       </c>
       <c r="I191" s="6"/>
     </row>
-    <row r="192" spans="2:9">
+    <row r="192" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B192" s="6"/>
       <c r="C192" s="5"/>
       <c r="D192" s="13"/>
@@ -5934,12 +5935,12 @@
       </c>
       <c r="I192" s="6"/>
     </row>
-    <row r="193" spans="7:8">
+    <row r="193" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G193" s="3"/>
       <c r="H193" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="B2:I180" xr:uid="{F75DB620-AF17-408B-81D4-431B9D551CF9}"/>
+  <autoFilter ref="B2:I192" xr:uid="{F75DB620-AF17-408B-81D4-431B9D551CF9}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>